<commit_message>
Add configurable file check verification rules
Introduce parent file-check configs with nested verification rules, exact-text search, validator reference dates, and compact JSON-backed rule configs in Excel.

Wire the checking UI for collapsible rule editing and add coverage for parsing, saving, and running verification checks.
</commit_message>
<xml_diff>
--- a/configuration-example.xlsx
+++ b/configuration-example.xlsx
@@ -8,20 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\kelvin\go\file-transfer\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{32A20F81-1143-40AF-9587-454C9774102A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11295"/>
   </bookViews>
   <sheets>
     <sheet name="File Transfers" sheetId="1" r:id="rId1"/>
     <sheet name="File Checks" sheetId="2" r:id="rId2"/>
+    <sheet name="File Check Rules" sheetId="3" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>Source Path</t>
   </si>
@@ -64,21 +64,66 @@
   <si>
     <t>D:\Reports\Daily\previous.xlsx</t>
   </si>
+  <si>
+    <t>Check ID</t>
+  </si>
+  <si>
+    <t>CHK-001</t>
+  </si>
+  <si>
+    <t>CHK-002</t>
+  </si>
+  <si>
+    <t>CHK-003</t>
+  </si>
+  <si>
+    <t>Rule ID</t>
+  </si>
+  <si>
+    <t>Rule Name</t>
+  </si>
+  <si>
+    <t>Rule Type</t>
+  </si>
+  <si>
+    <t>Enabled</t>
+  </si>
+  <si>
+    <t>Sheet</t>
+  </si>
+  <si>
+    <t>Anchor</t>
+  </si>
+  <si>
+    <t>Parent Direction</t>
+  </si>
+  <si>
+    <t>Header Depth</t>
+  </si>
+  <si>
+    <t>Require Order</t>
+  </si>
+  <si>
+    <t>Expected Text</t>
+  </si>
+  <si>
+    <t>Rule Config</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <fonts count="2">
     <font>
+      <name val="Carlito"/>
       <sz val="11"/>
-      <name val="Carlito"/>
     </font>
     <font>
-      <b/>
+      <name val="Carlito"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Carlito"/>
     </font>
   </fonts>
   <fills count="3">
@@ -108,18 +153,18 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true">
+      <alignment wrapText="true"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -132,7 +177,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ChatGPT">
   <a:themeElements>
     <a:clrScheme name="ChatGPT">
       <a:dk1>
@@ -281,13 +326,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="42" customWidth="1"/>
-    <col min="2" max="2" width="46" customWidth="1"/>
+    <col customWidth="true" max="1" min="1" width="42"/>
+    <col customWidth="true" max="2" min="2" width="46"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" ht="26.45" customHeight="true">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -295,7 +340,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="52.7" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="52.7" customHeight="true">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
@@ -303,7 +348,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="52.7" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="52.7" customHeight="true">
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
@@ -311,7 +356,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" ht="26.45" customHeight="true">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -327,45 +372,89 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="42" customWidth="1"/>
-    <col min="2" max="2" width="46" customWidth="1"/>
+    <col customWidth="true" max="2" min="2" width="42"/>
+    <col customWidth="true" max="3" min="3" width="46"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:2" ht="15" customHeight="true">
+      <c r="A1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="52.7" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:2" ht="52.7" customHeight="true">
+      <c r="A2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="66" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:2" ht="66" customHeight="true">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="52.7" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:2" ht="52.7" customHeight="true">
+      <c r="A4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>13</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <cols>
+    <col customWidth="true" max="5" min="1" width="18"/>
+    <col customWidth="true" max="6" min="6" width="72"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Redesign verification checks and inline editors
</commit_message>
<xml_diff>
--- a/configuration-example.xlsx
+++ b/configuration-example.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
   <si>
     <t>Source Path</t>
   </si>
@@ -108,6 +108,57 @@
   </si>
   <si>
     <t>Rule Config</t>
+  </si>
+  <si>
+    <t>SAMPLE-DEMO</t>
+  </si>
+  <si>
+    <t>sample/sample_file_05_31_2026.xlsx</t>
+  </si>
+  <si>
+    <t>sample/sample_file_04_30_2026.xlsx</t>
+  </si>
+  <si>
+    <t>TXT-001</t>
+  </si>
+  <si>
+    <t>Find sample text</t>
+  </si>
+  <si>
+    <t>exact_text</t>
+  </si>
+  <si>
+    <t>true</t>
+  </si>
+  <si>
+    <t>{"sheet":"Report","expected_text":"sometypeofTextthatneeds to be serached"}</t>
+  </si>
+  <si>
+    <t>HDR-001</t>
+  </si>
+  <si>
+    <t>Headers around date anchor</t>
+  </si>
+  <si>
+    <t>header_compare</t>
+  </si>
+  <si>
+    <t>{"sheet":"Report","anchor":"date","parent_direction":"up","max_header_depth":2,"require_order":true}</t>
+  </si>
+  <si>
+    <t>inception date anchor</t>
+  </si>
+  <si>
+    <t>File</t>
+  </si>
+  <si>
+    <t>Compare Offset Months</t>
+  </si>
+  <si>
+    <t>sample/sample_file_{mm}_{dd}_{yyyy}.xlsx</t>
+  </si>
+  <si>
+    <t>-1</t>
   </si>
 </sst>
 </file>
@@ -374,65 +425,10 @@
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col customWidth="true" max="2" min="2" width="42"/>
-    <col customWidth="true" max="3" min="3" width="46"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" ht="15" customHeight="true">
-      <c r="A1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" ht="52.7" customHeight="true">
-      <c r="A2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="66" customHeight="true">
-      <c r="A3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="52.7" customHeight="true">
-      <c r="A4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1"/>
-  <cols>
-    <col customWidth="true" max="5" min="1" width="18"/>
-    <col customWidth="true" max="6" min="6" width="72"/>
+    <col customWidth="true" max="1" min="1" width="24"/>
+    <col customWidth="true" max="2" min="2" width="54"/>
+    <col customWidth="true" max="3" min="3" width="24"/>
+    <col customWidth="true" max="6" min="4" width="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -440,6 +436,41 @@
         <v>14</v>
       </c>
       <c r="B1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <cols>
+    <col customWidth="true" max="5" min="1" width="20"/>
+    <col customWidth="true" max="6" min="6" width="96"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" t="s">
         <v>18</v>
       </c>
       <c r="C1" t="s">
@@ -453,6 +484,46 @@
       </c>
       <c r="F1" t="s">
         <v>28</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D3" t="s">
+        <v>39</v>
+      </c>
+      <c r="E3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F3" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Expand sample verification workbook
</commit_message>
<xml_diff>
--- a/configuration-example.xlsx
+++ b/configuration-example.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
   <si>
     <t>Source Path</t>
   </si>
@@ -159,6 +159,24 @@
   </si>
   <si>
     <t>-1</t>
+  </si>
+  <si>
+    <t>{"sheet":"Report","anchor":"date","parent_direction":"up","max_header_depth":3,"require_order":true}</t>
+  </si>
+  <si>
+    <t>SCAN-001</t>
+  </si>
+  <si>
+    <t>Reporting date scan</t>
+  </si>
+  <si>
+    <t>anchor_scan_match</t>
+  </si>
+  <si>
+    <t>{"sheet":"Report","anchor":"Reporting dates","direction":"down","select":"last_non_empty_before_blank","expected_text":"{mm}/{dd}/{yy}","compare_as":"date"}</t>
+  </si>
+  <si>
+    <t>sample/sample_file_{mm}_*_{yyyy}.xlsx</t>
   </si>
 </sst>
 </file>
@@ -447,7 +465,7 @@
         <v>29</v>
       </c>
       <c r="B2" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="C2" t="s">
         <v>45</v>
@@ -514,7 +532,7 @@
         <v>37</v>
       </c>
       <c r="C3" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D3" t="s">
         <v>39</v>
@@ -523,7 +541,27 @@
         <v>35</v>
       </c>
       <c r="F3" t="s">
-        <v>40</v>
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D4" t="s">
+        <v>49</v>
+      </c>
+      <c r="E4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F4" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>